<commit_message>
8~10월(2026_03) 보정 — 5~7월 실측 반영
- 5~7월 실측(연금 7.6억·IRP 1.8억)으로 3가지 보정:
  ① 신청 스케일 δ=0.783(모델 대비 실측 1.28배 과대) ② IRP 비중 24% ③ 지급률32.5%·리워드12.77만 유지(검증됨)
- 8~10월 보정 예산: 연금 기준 6.80억(기존 8.68→-22%), IRP 기준 1.61억(기존 5.49→-71%), 합계 기준 8.40억
- 낙관 10.51억 / MC 연금 P90 8.99억(합계 P90 ≈ 11.1억) — 5~7월이 낙관 실현된 점 반영해 상단 편성 권고
- Excel '보정_8_10월' 시트 추가

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Rf55wZTokShwEgBjoVPEd8
</commit_message>
<xml_diff>
--- a/reports/연금저축_이벤트_시뮬레이션_보고서.xlsx
+++ b/reports/연금저축_이벤트_시뮬레이션_보고서.xlsx
@@ -12,8 +12,9 @@
     <sheet name="방법론_상세" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Nowcast_5_7월" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="향후회차예측" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="몬테카를로" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="참고실적" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="보정_8_10월" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="몬테카를로" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="참고실적" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -157,7 +158,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -265,6 +266,9 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="173" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -1922,6 +1926,237 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>8~10월(2026_03) 보정 — 5~7월 실측 반영</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="35" t="inlineStr">
+        <is>
+          <t>5~7월 실측(연금 7.6억·IRP 1.8억)으로 3가지 보정:</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="35" t="inlineStr">
+        <is>
+          <t>① 신청 스케일: 모델이 실측 대비 1.28배 과대 → 보정계수 δ=0.783 적용(신청 하향).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>② IRP 비중: 실측 IRP/연금 = 24% 반영(기존 과대 → 대폭 하향).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="35" t="inlineStr">
+        <is>
+          <t>③ 지급률 32.5%·리워드 12.7665만원: 5~7월에서 검증됨 → 유지.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="35" t="inlineStr">
+        <is>
+          <t>※ 5~7월 실제가 낙관(상단)에서 실현(마감 급증) → 편성은 낙관/P90 권고.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>시나리오</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>연금 신청(보정)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>연금 예산</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>IRP 예산</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>합계</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>보수</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>12292</v>
+      </c>
+      <c r="C9" s="36" t="n">
+        <v>5.0998957363575</v>
+      </c>
+      <c r="D9" s="36" t="n">
+        <v>1.208675289516727</v>
+      </c>
+      <c r="E9" s="36" t="n">
+        <v>6.308571025874228</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>기준</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>16388</v>
+      </c>
+      <c r="C10" s="36" t="n">
+        <v>6.799644398137501</v>
+      </c>
+      <c r="D10" s="36" t="n">
+        <v>1.611515722358588</v>
+      </c>
+      <c r="E10" s="39" t="n">
+        <v>8.411160120496088</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>낙관</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>20486</v>
+      </c>
+      <c r="C11" s="36" t="n">
+        <v>8.499717935426251</v>
+      </c>
+      <c r="D11" s="36" t="n">
+        <v>2.014433150696021</v>
+      </c>
+      <c r="E11" s="36" t="n">
+        <v>10.51415108612227</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>[ 몬테카를로 (보정 take-rate, 지급률 Beta CV 0.22) — 연금 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>구분</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>P50</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>P90(권고)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>P95</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>연금 8~10월</t>
+        </is>
+      </c>
+      <c r="B15" s="36" t="n">
+        <v>6.68</v>
+      </c>
+      <c r="C15" s="37" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="D15" s="36" t="n">
+        <v>9.69</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="35" t="inlineStr">
+        <is>
+          <t>합계(+IRP 24%) P90 ≈ 11.1억</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>[ 기존(보정 전) 대비 ]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="35" t="inlineStr">
+        <is>
+          <t>연금 기준 8.68억 → 6.80억(-22%) · IRP 기준 5.49억 → 1.61억(-71%, 비중 재보정)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="35" t="inlineStr">
+        <is>
+          <t>합계 기준 8.40억 · 낙관 10.51억 · MC P90(합계) ≈ 11.1억</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="9">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A20:E20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A16:E16"/>
+    <mergeCell ref="A19:E19"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A6:E6"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2140,8 +2375,8 @@
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A4:E4"/>
     <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A5:E5"/>
     <mergeCell ref="A17:E17"/>
     <mergeCell ref="A3:E3"/>
   </mergeCells>
@@ -2149,7 +2384,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>